<commit_message>
Run 1 is complete
</commit_message>
<xml_diff>
--- a/simrun_results_pretty.xlsx
+++ b/simrun_results_pretty.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ian\git\REVASC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4A17188-524A-41A2-B9B7-30B30B3D296B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD681C9E-9BD2-4C8E-A717-C40F44643540}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="42690" yWindow="15" windowWidth="15015" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="21615" windowHeight="20985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="run 2" sheetId="1" r:id="rId1"/>
+    <sheet name="run 1" sheetId="2" r:id="rId1"/>
+    <sheet name="run 2" sheetId="1" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -33,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="25">
   <si>
     <t>N_tot</t>
   </si>
@@ -106,6 +107,9 @@
   <si>
     <t>FWER</t>
   </si>
+  <si>
+    <t>Cl7</t>
+  </si>
 </sst>
 </file>
 
@@ -159,7 +163,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -185,17 +189,23 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -501,18 +511,17 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L36"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{06007A61-CD46-4A24-8404-A842DC1469EA}">
+  <dimension ref="A1:M36"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.7265625" style="1"/>
-    <col min="2" max="4" width="8.7265625" style="6"/>
-    <col min="5" max="11" width="8.7265625" style="7"/>
-    <col min="12" max="12" width="11.54296875" style="11" bestFit="1" customWidth="1"/>
-    <col min="13" max="16384" width="8.7265625" style="6"/>
+    <col min="1" max="1" width="10.7109375" style="1" customWidth="1"/>
+    <col min="2" max="3" width="10.7109375" customWidth="1"/>
+    <col min="4" max="4" width="10.7109375" style="6" customWidth="1"/>
+    <col min="5" max="13" width="10.7109375" style="13" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:13" s="2" customFormat="1" ht="45" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>8</v>
       </c>
@@ -525,62 +534,1154 @@
       <c r="D1" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="G1" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="H1" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="I1" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="J1" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="K1" s="3" t="s">
+      <c r="K1" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="L1" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="L1" s="9" t="s">
+      <c r="M1" s="9" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1"/>
       <c r="D2" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="E2" s="4">
-        <v>0.25287808000000001</v>
-      </c>
-      <c r="F2" s="4">
-        <v>7.4864760000000002E-2</v>
-      </c>
-      <c r="G2" s="4">
-        <v>0.28325396000000003</v>
-      </c>
-      <c r="H2" s="4">
-        <v>0.26791576</v>
-      </c>
-      <c r="I2" s="4">
-        <v>7.1119790000000002E-2</v>
-      </c>
-      <c r="J2" s="4">
-        <v>4.9967640000000001E-2</v>
-      </c>
-      <c r="K2" s="3"/>
-      <c r="L2" s="10"/>
-    </row>
-    <row r="3" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="E2" s="11">
+        <v>0.25</v>
+      </c>
+      <c r="F2" s="11">
+        <v>0.04</v>
+      </c>
+      <c r="G2" s="11">
+        <v>0.06</v>
+      </c>
+      <c r="H2" s="11">
+        <v>0.27</v>
+      </c>
+      <c r="I2" s="11">
+        <v>0.24</v>
+      </c>
+      <c r="J2" s="11">
+        <v>0.09</v>
+      </c>
+      <c r="K2" s="11">
+        <v>0.05</v>
+      </c>
+      <c r="L2" s="3"/>
+      <c r="M2" s="3"/>
+    </row>
+    <row r="3" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="D3" s="3" t="s">
         <v>12</v>
       </c>
+      <c r="E3" s="11">
+        <v>0.623</v>
+      </c>
+      <c r="F3" s="11">
+        <v>0.49</v>
+      </c>
+      <c r="G3" s="11">
+        <v>0.39800000000000002</v>
+      </c>
+      <c r="H3" s="11">
+        <v>0.60899999999999999</v>
+      </c>
+      <c r="I3" s="11">
+        <v>0.39200000000000002</v>
+      </c>
+      <c r="J3" s="11">
+        <v>0.72</v>
+      </c>
+      <c r="K3" s="11">
+        <v>0.68899999999999995</v>
+      </c>
+      <c r="L3" s="3"/>
+      <c r="M3" s="3"/>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A4" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="E4" s="12"/>
+      <c r="F4" s="12"/>
+      <c r="G4" s="12"/>
+      <c r="H4" s="12"/>
+      <c r="I4" s="12"/>
+      <c r="J4" s="12"/>
+      <c r="K4" s="12"/>
+      <c r="L4" s="12"/>
+      <c r="M4" s="12"/>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="B5">
+        <v>1500</v>
+      </c>
+      <c r="C5">
+        <v>5000</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="E5" s="14">
+        <v>2.5600000000000001E-2</v>
+      </c>
+      <c r="F5" s="14">
+        <v>2.3599999999999999E-2</v>
+      </c>
+      <c r="G5" s="14">
+        <v>2.2599999999999999E-2</v>
+      </c>
+      <c r="H5" s="14">
+        <v>2.4799999999999999E-2</v>
+      </c>
+      <c r="I5" s="14">
+        <v>2.8000000000000001E-2</v>
+      </c>
+      <c r="J5" s="14">
+        <v>2.3599999999999999E-2</v>
+      </c>
+      <c r="K5" s="14">
+        <v>2.1600000000000001E-2</v>
+      </c>
+      <c r="L5" s="14">
+        <v>0.15840000000000001</v>
+      </c>
+      <c r="M5" s="14"/>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="B6">
+        <v>1500</v>
+      </c>
+      <c r="C6">
+        <v>5000</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="E6" s="14">
+        <v>1.18E-2</v>
+      </c>
+      <c r="F6" s="14">
+        <v>5.9999999999999995E-4</v>
+      </c>
+      <c r="G6" s="14">
+        <v>1.8E-3</v>
+      </c>
+      <c r="H6" s="14">
+        <v>1.0999999999999999E-2</v>
+      </c>
+      <c r="I6" s="14">
+        <v>7.0000000000000001E-3</v>
+      </c>
+      <c r="J6" s="14">
+        <v>4.4000000000000003E-3</v>
+      </c>
+      <c r="K6" s="14">
+        <v>1.1999999999999999E-3</v>
+      </c>
+      <c r="L6" s="14">
+        <v>2.7199999999999998E-2</v>
+      </c>
+      <c r="M6" s="14"/>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A7" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="E7" s="14"/>
+      <c r="F7" s="14"/>
+      <c r="G7" s="14"/>
+      <c r="H7" s="14"/>
+      <c r="I7" s="14"/>
+      <c r="J7" s="14"/>
+      <c r="K7" s="14"/>
+      <c r="L7" s="14"/>
+      <c r="M7" s="14"/>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="B8">
+        <v>1500</v>
+      </c>
+      <c r="C8">
+        <v>5000</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="E8" s="14">
+        <v>0.62560000000000004</v>
+      </c>
+      <c r="F8" s="14">
+        <v>0.10920000000000001</v>
+      </c>
+      <c r="G8" s="14">
+        <v>0.1226</v>
+      </c>
+      <c r="H8" s="14">
+        <v>0.62180000000000002</v>
+      </c>
+      <c r="I8" s="14">
+        <v>0.4204</v>
+      </c>
+      <c r="J8" s="14">
+        <v>0.30559999999999998</v>
+      </c>
+      <c r="K8" s="14">
+        <v>0.17760000000000001</v>
+      </c>
+      <c r="L8" s="14">
+        <v>0</v>
+      </c>
+      <c r="M8" s="14">
+        <v>0.47328999999999999</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="B9">
+        <v>1500</v>
+      </c>
+      <c r="C9">
+        <v>5000</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="E9" s="14">
+        <v>0.86599999999999999</v>
+      </c>
+      <c r="F9" s="14">
+        <v>0.47560000000000002</v>
+      </c>
+      <c r="G9" s="14">
+        <v>0.50460000000000005</v>
+      </c>
+      <c r="H9" s="14">
+        <v>0.85940000000000005</v>
+      </c>
+      <c r="I9" s="14">
+        <v>0.75700000000000001</v>
+      </c>
+      <c r="J9" s="14">
+        <v>0.69440000000000002</v>
+      </c>
+      <c r="K9" s="14">
+        <v>0.56999999999999995</v>
+      </c>
+      <c r="L9" s="14">
+        <v>0</v>
+      </c>
+      <c r="M9" s="14">
+        <v>0.77051400000000003</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="E10" s="14"/>
+      <c r="F10" s="14"/>
+      <c r="G10" s="14"/>
+      <c r="H10" s="14"/>
+      <c r="I10" s="14"/>
+      <c r="J10" s="14"/>
+      <c r="K10" s="14"/>
+      <c r="L10" s="14"/>
+      <c r="M10" s="14"/>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="B11">
+        <v>2000</v>
+      </c>
+      <c r="C11">
+        <v>5000</v>
+      </c>
+      <c r="D11" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="E11" s="14">
+        <v>0.74439999999999995</v>
+      </c>
+      <c r="F11" s="14">
+        <v>0.13919999999999999</v>
+      </c>
+      <c r="G11" s="14">
+        <v>0.157</v>
+      </c>
+      <c r="H11" s="14">
+        <v>0.7762</v>
+      </c>
+      <c r="I11" s="14">
+        <v>0.52900000000000003</v>
+      </c>
+      <c r="J11" s="14">
+        <v>0.38940000000000002</v>
+      </c>
+      <c r="K11" s="14">
+        <v>0.23</v>
+      </c>
+      <c r="L11" s="14">
+        <v>0</v>
+      </c>
+      <c r="M11" s="14">
+        <v>0.58416800000000002</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="B12">
+        <v>2000</v>
+      </c>
+      <c r="C12">
+        <v>5000</v>
+      </c>
+      <c r="D12" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="E12" s="14">
+        <v>0.92900000000000005</v>
+      </c>
+      <c r="F12" s="14">
+        <v>0.59379999999999999</v>
+      </c>
+      <c r="G12" s="14">
+        <v>0.62639999999999996</v>
+      </c>
+      <c r="H12" s="14">
+        <v>0.93820000000000003</v>
+      </c>
+      <c r="I12" s="14">
+        <v>0.86140000000000005</v>
+      </c>
+      <c r="J12" s="14">
+        <v>0.7974</v>
+      </c>
+      <c r="K12" s="14">
+        <v>0.68540000000000001</v>
+      </c>
+      <c r="L12" s="14">
+        <v>0</v>
+      </c>
+      <c r="M12" s="14">
+        <v>0.8596720000000001</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="E13" s="14"/>
+      <c r="F13" s="14"/>
+      <c r="G13" s="14"/>
+      <c r="H13" s="14"/>
+      <c r="I13" s="14"/>
+      <c r="J13" s="14"/>
+      <c r="K13" s="14"/>
+      <c r="L13" s="14"/>
+      <c r="M13" s="14"/>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="B14">
+        <v>2500</v>
+      </c>
+      <c r="C14">
+        <v>5000</v>
+      </c>
+      <c r="D14" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="E14" s="14">
+        <v>0.83199999999999996</v>
+      </c>
+      <c r="F14" s="14">
+        <v>0.16719999999999999</v>
+      </c>
+      <c r="G14" s="14">
+        <v>0.1996</v>
+      </c>
+      <c r="H14" s="14">
+        <v>0.84699999999999998</v>
+      </c>
+      <c r="I14" s="14">
+        <v>0.60919999999999996</v>
+      </c>
+      <c r="J14" s="14">
+        <v>0.47420000000000001</v>
+      </c>
+      <c r="K14" s="14">
+        <v>0.2712</v>
+      </c>
+      <c r="L14" s="14">
+        <v>0</v>
+      </c>
+      <c r="M14" s="14">
+        <v>0.65779999999999994</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="B15">
+        <v>2500</v>
+      </c>
+      <c r="C15">
+        <v>5000</v>
+      </c>
+      <c r="D15" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="E15" s="14">
+        <v>0.96160000000000001</v>
+      </c>
+      <c r="F15" s="14">
+        <v>0.68879999999999997</v>
+      </c>
+      <c r="G15" s="14">
+        <v>0.70740000000000003</v>
+      </c>
+      <c r="H15" s="14">
+        <v>0.96899999999999997</v>
+      </c>
+      <c r="I15" s="14">
+        <v>0.90180000000000005</v>
+      </c>
+      <c r="J15" s="14">
+        <v>0.8468</v>
+      </c>
+      <c r="K15" s="14">
+        <v>0.76259999999999994</v>
+      </c>
+      <c r="L15" s="14">
+        <v>0</v>
+      </c>
+      <c r="M15" s="14">
+        <v>0.90280000000000005</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="E16" s="14"/>
+      <c r="F16" s="14"/>
+      <c r="G16" s="14"/>
+      <c r="H16" s="14"/>
+      <c r="I16" s="14"/>
+      <c r="J16" s="14"/>
+      <c r="K16" s="14"/>
+      <c r="L16" s="14"/>
+      <c r="M16" s="14"/>
+    </row>
+    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="B17">
+        <v>3000</v>
+      </c>
+      <c r="C17">
+        <v>5000</v>
+      </c>
+      <c r="D17" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="E17" s="14">
+        <v>0.88839999999999997</v>
+      </c>
+      <c r="F17" s="14">
+        <v>0.2014</v>
+      </c>
+      <c r="G17" s="14">
+        <v>0.2384</v>
+      </c>
+      <c r="H17" s="14">
+        <v>0.90659999999999996</v>
+      </c>
+      <c r="I17" s="14">
+        <v>0.69599999999999995</v>
+      </c>
+      <c r="J17" s="14">
+        <v>0.53100000000000003</v>
+      </c>
+      <c r="K17" s="14">
+        <v>0.3246</v>
+      </c>
+      <c r="L17" s="14">
+        <v>0</v>
+      </c>
+      <c r="M17" s="14">
+        <v>0.720302</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="B18">
+        <v>3000</v>
+      </c>
+      <c r="C18">
+        <v>5000</v>
+      </c>
+      <c r="D18" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="E18" s="14">
+        <v>0.98280000000000001</v>
+      </c>
+      <c r="F18" s="14">
+        <v>0.752</v>
+      </c>
+      <c r="G18" s="14">
+        <v>0.76780000000000004</v>
+      </c>
+      <c r="H18" s="14">
+        <v>0.98399999999999999</v>
+      </c>
+      <c r="I18" s="14">
+        <v>0.93940000000000001</v>
+      </c>
+      <c r="J18" s="14">
+        <v>0.89459999999999995</v>
+      </c>
+      <c r="K18" s="14">
+        <v>0.83099999999999996</v>
+      </c>
+      <c r="L18" s="14">
+        <v>0</v>
+      </c>
+      <c r="M18" s="14">
+        <v>0.93504799999999999</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A19" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E19" s="14"/>
+      <c r="F19" s="14"/>
+      <c r="G19" s="14"/>
+      <c r="H19" s="14"/>
+      <c r="I19" s="14"/>
+      <c r="J19" s="14"/>
+      <c r="K19" s="14"/>
+      <c r="L19" s="14"/>
+      <c r="M19" s="14"/>
+    </row>
+    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="B20">
+        <v>3000</v>
+      </c>
+      <c r="C20">
+        <v>5000</v>
+      </c>
+      <c r="D20" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="E20" s="14">
+        <v>0.89100000000000001</v>
+      </c>
+      <c r="F20" s="14">
+        <v>2.2599999999999999E-2</v>
+      </c>
+      <c r="G20" s="14">
+        <v>0.23680000000000001</v>
+      </c>
+      <c r="H20" s="14">
+        <v>0.90839999999999999</v>
+      </c>
+      <c r="I20" s="14">
+        <v>0.69340000000000002</v>
+      </c>
+      <c r="J20" s="14">
+        <v>0.54259999999999997</v>
+      </c>
+      <c r="K20" s="14">
+        <v>0.31259999999999999</v>
+      </c>
+      <c r="L20" s="14">
+        <v>2.2599999999999999E-2</v>
+      </c>
+      <c r="M20" s="14">
+        <v>0.74281875000000008</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="B21">
+        <v>3000</v>
+      </c>
+      <c r="C21">
+        <v>5000</v>
+      </c>
+      <c r="D21" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="E21" s="14">
+        <v>0.9778</v>
+      </c>
+      <c r="F21" s="14">
+        <v>0.374</v>
+      </c>
+      <c r="G21" s="14">
+        <v>0.70199999999999996</v>
+      </c>
+      <c r="H21" s="14">
+        <v>0.97760000000000002</v>
+      </c>
+      <c r="I21" s="14">
+        <v>0.91639999999999999</v>
+      </c>
+      <c r="J21" s="14">
+        <v>0.87160000000000004</v>
+      </c>
+      <c r="K21" s="14">
+        <v>0.76419999999999999</v>
+      </c>
+      <c r="L21" s="14">
+        <v>0.374</v>
+      </c>
+      <c r="M21" s="14">
+        <v>0.92407500000000009</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A22" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="E22" s="14"/>
+      <c r="F22" s="14"/>
+      <c r="G22" s="14"/>
+      <c r="H22" s="14"/>
+      <c r="I22" s="14"/>
+      <c r="J22" s="14"/>
+      <c r="K22" s="14"/>
+      <c r="L22" s="14"/>
+      <c r="M22" s="14"/>
+    </row>
+    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="B23">
+        <v>3000</v>
+      </c>
+      <c r="C23">
+        <v>5000</v>
+      </c>
+      <c r="D23" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="E23" s="14">
+        <v>0.89100000000000001</v>
+      </c>
+      <c r="F23" s="14">
+        <v>0.18579999999999999</v>
+      </c>
+      <c r="G23" s="14">
+        <v>0.22919999999999999</v>
+      </c>
+      <c r="H23" s="14">
+        <v>2.1000000000000001E-2</v>
+      </c>
+      <c r="I23" s="14">
+        <v>0.7006</v>
+      </c>
+      <c r="J23" s="14">
+        <v>0.53820000000000001</v>
+      </c>
+      <c r="K23" s="14">
+        <v>0.31480000000000002</v>
+      </c>
+      <c r="L23" s="14">
+        <v>2.1000000000000001E-2</v>
+      </c>
+      <c r="M23" s="14">
+        <v>0.65240547945205485</v>
+      </c>
+    </row>
+    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="B24">
+        <v>3000</v>
+      </c>
+      <c r="C24">
+        <v>5000</v>
+      </c>
+      <c r="D24" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="E24" s="14">
+        <v>0.94540000000000002</v>
+      </c>
+      <c r="F24" s="14">
+        <v>0.34520000000000001</v>
+      </c>
+      <c r="G24" s="14">
+        <v>0.41</v>
+      </c>
+      <c r="H24" s="14">
+        <v>0.11459999999999999</v>
+      </c>
+      <c r="I24" s="14">
+        <v>0.83899999999999997</v>
+      </c>
+      <c r="J24" s="14">
+        <v>0.72340000000000004</v>
+      </c>
+      <c r="K24" s="14">
+        <v>0.52300000000000002</v>
+      </c>
+      <c r="L24" s="14">
+        <v>0.11459999999999999</v>
+      </c>
+      <c r="M24" s="14">
+        <v>0.77722465753424652</v>
+      </c>
+    </row>
+    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A25" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="E25" s="14"/>
+      <c r="F25" s="14"/>
+      <c r="G25" s="14"/>
+      <c r="H25" s="14"/>
+      <c r="I25" s="14"/>
+      <c r="J25" s="14"/>
+      <c r="K25" s="14"/>
+      <c r="L25" s="14"/>
+      <c r="M25" s="14"/>
+    </row>
+    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="B26">
+        <v>3000</v>
+      </c>
+      <c r="C26">
+        <v>5000</v>
+      </c>
+      <c r="D26" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="E26" s="14">
+        <v>2.58E-2</v>
+      </c>
+      <c r="F26" s="14">
+        <v>0.20219999999999999</v>
+      </c>
+      <c r="G26" s="14">
+        <v>2.5399999999999999E-2</v>
+      </c>
+      <c r="H26" s="14">
+        <v>2.5000000000000001E-2</v>
+      </c>
+      <c r="I26" s="14">
+        <v>2.2200000000000001E-2</v>
+      </c>
+      <c r="J26" s="14">
+        <v>2.6800000000000001E-2</v>
+      </c>
+      <c r="K26" s="14">
+        <v>2.4E-2</v>
+      </c>
+      <c r="L26" s="14">
+        <v>0.1384</v>
+      </c>
+      <c r="M26" s="14">
+        <v>0.20219999999999999</v>
+      </c>
+    </row>
+    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="B27">
+        <v>3000</v>
+      </c>
+      <c r="C27">
+        <v>5000</v>
+      </c>
+      <c r="D27" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="E27" s="14">
+        <v>1.6400000000000001E-2</v>
+      </c>
+      <c r="F27" s="14">
+        <v>7.1999999999999998E-3</v>
+      </c>
+      <c r="G27" s="14">
+        <v>1.6000000000000001E-3</v>
+      </c>
+      <c r="H27" s="14">
+        <v>1.72E-2</v>
+      </c>
+      <c r="I27" s="14">
+        <v>8.6E-3</v>
+      </c>
+      <c r="J27" s="14">
+        <v>8.8000000000000005E-3</v>
+      </c>
+      <c r="K27" s="14">
+        <v>3.8E-3</v>
+      </c>
+      <c r="L27" s="14">
+        <v>4.4600000000000001E-2</v>
+      </c>
+      <c r="M27" s="14">
+        <v>7.1999999999999998E-3</v>
+      </c>
+    </row>
+    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A28" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="E28" s="14"/>
+      <c r="F28" s="14"/>
+      <c r="G28" s="14"/>
+      <c r="H28" s="14"/>
+      <c r="I28" s="14"/>
+      <c r="J28" s="14"/>
+      <c r="K28" s="14"/>
+      <c r="L28" s="14"/>
+      <c r="M28" s="14"/>
+    </row>
+    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="B29">
+        <v>3000</v>
+      </c>
+      <c r="C29">
+        <v>5000</v>
+      </c>
+      <c r="D29" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="E29" s="14">
+        <v>2.5000000000000001E-2</v>
+      </c>
+      <c r="F29" s="14">
+        <v>2.76E-2</v>
+      </c>
+      <c r="G29" s="14">
+        <v>2.46E-2</v>
+      </c>
+      <c r="H29" s="14">
+        <v>0.90039999999999998</v>
+      </c>
+      <c r="I29" s="14">
+        <v>2.5000000000000001E-2</v>
+      </c>
+      <c r="J29" s="14">
+        <v>2.8400000000000002E-2</v>
+      </c>
+      <c r="K29" s="14">
+        <v>2.6800000000000001E-2</v>
+      </c>
+      <c r="L29" s="14">
+        <v>0.1484</v>
+      </c>
+      <c r="M29" s="14">
+        <v>0.90039999999999998</v>
+      </c>
+    </row>
+    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="B30">
+        <v>3000</v>
+      </c>
+      <c r="C30">
+        <v>5000</v>
+      </c>
+      <c r="D30" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="E30" s="14">
+        <v>3.8399999999999997E-2</v>
+      </c>
+      <c r="F30" s="14">
+        <v>8.2000000000000007E-3</v>
+      </c>
+      <c r="G30" s="14">
+        <v>1.24E-2</v>
+      </c>
+      <c r="H30" s="14">
+        <v>0.77039999999999997</v>
+      </c>
+      <c r="I30" s="14">
+        <v>3.04E-2</v>
+      </c>
+      <c r="J30" s="14">
+        <v>2.8199999999999999E-2</v>
+      </c>
+      <c r="K30" s="14">
+        <v>1.4800000000000001E-2</v>
+      </c>
+      <c r="L30" s="14">
+        <v>0.1026</v>
+      </c>
+      <c r="M30" s="14">
+        <v>0.77039999999999997</v>
+      </c>
+    </row>
+    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A31" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E31" s="14"/>
+      <c r="F31" s="14"/>
+      <c r="G31" s="14"/>
+      <c r="H31" s="14"/>
+      <c r="I31" s="14"/>
+      <c r="J31" s="14"/>
+      <c r="K31" s="14"/>
+      <c r="L31" s="14"/>
+      <c r="M31" s="14"/>
+    </row>
+    <row r="32" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="B32">
+        <v>3000</v>
+      </c>
+      <c r="C32">
+        <v>5000</v>
+      </c>
+      <c r="D32" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="E32" s="14">
+        <v>2.6800000000000001E-2</v>
+      </c>
+      <c r="F32" s="14">
+        <v>0.2</v>
+      </c>
+      <c r="G32" s="14">
+        <v>0.2326</v>
+      </c>
+      <c r="H32" s="14">
+        <v>2.5999999999999999E-2</v>
+      </c>
+      <c r="I32" s="14">
+        <v>2.4199999999999999E-2</v>
+      </c>
+      <c r="J32" s="14">
+        <v>0.54779999999999995</v>
+      </c>
+      <c r="K32" s="14">
+        <v>0.312</v>
+      </c>
+      <c r="L32" s="14">
+        <v>7.4999999999999997E-2</v>
+      </c>
+      <c r="M32" s="14">
+        <v>0.36190833333333328</v>
+      </c>
+    </row>
+    <row r="33" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="B33">
+        <v>3000</v>
+      </c>
+      <c r="C33">
+        <v>5000</v>
+      </c>
+      <c r="D33" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="E33" s="14">
+        <v>5.1999999999999998E-2</v>
+      </c>
+      <c r="F33" s="14">
+        <v>9.6600000000000005E-2</v>
+      </c>
+      <c r="G33" s="14">
+        <v>0.12659999999999999</v>
+      </c>
+      <c r="H33" s="14">
+        <v>4.7600000000000003E-2</v>
+      </c>
+      <c r="I33" s="14">
+        <v>4.58E-2</v>
+      </c>
+      <c r="J33" s="14">
+        <v>0.42920000000000003</v>
+      </c>
+      <c r="K33" s="14">
+        <v>0.2152</v>
+      </c>
+      <c r="L33" s="14">
+        <v>0.1222</v>
+      </c>
+      <c r="M33" s="14">
+        <v>0.25353333333333328</v>
+      </c>
+    </row>
+    <row r="34" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A34" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="E34" s="14"/>
+      <c r="F34" s="14"/>
+      <c r="G34" s="14"/>
+      <c r="H34" s="14"/>
+      <c r="I34" s="14"/>
+      <c r="J34" s="14"/>
+      <c r="K34" s="14"/>
+      <c r="L34" s="14"/>
+      <c r="M34" s="14"/>
+    </row>
+    <row r="35" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="B35">
+        <v>3000</v>
+      </c>
+      <c r="C35">
+        <v>5000</v>
+      </c>
+      <c r="D35" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="E35" s="14">
+        <v>0.89680000000000004</v>
+      </c>
+      <c r="F35" s="14">
+        <v>2.2200000000000001E-2</v>
+      </c>
+      <c r="G35" s="14">
+        <v>2.3E-2</v>
+      </c>
+      <c r="H35" s="14">
+        <v>0.91339999999999999</v>
+      </c>
+      <c r="I35" s="14">
+        <v>0.68740000000000001</v>
+      </c>
+      <c r="J35" s="14">
+        <v>2.58E-2</v>
+      </c>
+      <c r="K35" s="14">
+        <v>2.4199999999999999E-2</v>
+      </c>
+      <c r="L35" s="14">
+        <v>9.0800000000000006E-2</v>
+      </c>
+      <c r="M35" s="14">
+        <v>0.83657105263157894</v>
+      </c>
+    </row>
+    <row r="36" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="B36">
+        <v>3000</v>
+      </c>
+      <c r="C36">
+        <v>5000</v>
+      </c>
+      <c r="D36" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="E36" s="14">
+        <v>0.93859999999999999</v>
+      </c>
+      <c r="F36" s="14">
+        <v>7.8200000000000006E-2</v>
+      </c>
+      <c r="G36" s="14">
+        <v>8.9399999999999993E-2</v>
+      </c>
+      <c r="H36" s="14">
+        <v>0.95499999999999996</v>
+      </c>
+      <c r="I36" s="14">
+        <v>0.79020000000000001</v>
+      </c>
+      <c r="J36" s="14">
+        <v>0.1028</v>
+      </c>
+      <c r="K36" s="14">
+        <v>9.98E-2</v>
+      </c>
+      <c r="L36" s="14">
+        <v>0.24579999999999999</v>
+      </c>
+      <c r="M36" s="14">
+        <v>0.89756315789473684</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:L36"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="10.7109375" style="1" customWidth="1"/>
+    <col min="2" max="4" width="10.7109375" style="6" customWidth="1"/>
+    <col min="5" max="12" width="10.7109375" style="7" customWidth="1"/>
+    <col min="13" max="16384" width="8.7109375" style="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12" s="2" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="K1" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="L1" s="9" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="1"/>
+      <c r="D2" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E2" s="4">
+        <v>0.25287808000000001</v>
+      </c>
+      <c r="F2" s="4">
+        <v>7.4864760000000002E-2</v>
+      </c>
+      <c r="G2" s="4">
+        <v>0.28325396000000003</v>
+      </c>
+      <c r="H2" s="4">
+        <v>0.26791576</v>
+      </c>
+      <c r="I2" s="4">
+        <v>7.1119790000000002E-2</v>
+      </c>
+      <c r="J2" s="4">
+        <v>4.9967640000000001E-2</v>
+      </c>
+      <c r="K2" s="3"/>
+      <c r="L2" s="3"/>
+    </row>
+    <row r="3" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="1"/>
+      <c r="D3" s="3" t="s">
+        <v>12</v>
+      </c>
       <c r="E3" s="4">
         <v>0.60697330000000005</v>
       </c>
@@ -600,14 +1701,14 @@
         <v>0.67542860000000005</v>
       </c>
       <c r="K3" s="3"/>
-      <c r="L3" s="10"/>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="L3" s="3"/>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B5" s="6">
         <v>1500</v>
       </c>
@@ -638,9 +1739,9 @@
       <c r="K5" s="8">
         <v>0.13600000000000001</v>
       </c>
-      <c r="L5" s="12"/>
-    </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="L5" s="10"/>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B6" s="6">
         <v>1500</v>
       </c>
@@ -671,9 +1772,9 @@
       <c r="K6" s="8">
         <v>3.1E-2</v>
       </c>
-      <c r="L6" s="12"/>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="L6" s="10"/>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
         <v>10</v>
       </c>
@@ -684,9 +1785,9 @@
       <c r="I7" s="8"/>
       <c r="J7" s="8"/>
       <c r="K7" s="8"/>
-      <c r="L7" s="12"/>
-    </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="L7" s="10"/>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B8" s="6">
         <v>1500</v>
       </c>
@@ -717,11 +1818,11 @@
       <c r="K8" s="8">
         <v>0</v>
       </c>
-      <c r="L8" s="12">
+      <c r="L8" s="10">
         <v>0.49386085348374859</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B9" s="6">
         <v>1500</v>
       </c>
@@ -752,11 +1853,11 @@
       <c r="K9" s="8">
         <v>0</v>
       </c>
-      <c r="L9" s="12">
+      <c r="L9" s="10">
         <v>0.77324196911553933</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="E10" s="8"/>
       <c r="F10" s="8"/>
       <c r="G10" s="8"/>
@@ -764,9 +1865,9 @@
       <c r="I10" s="8"/>
       <c r="J10" s="8"/>
       <c r="K10" s="8"/>
-      <c r="L10" s="12"/>
-    </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="L10" s="10"/>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B11" s="6">
         <v>2000</v>
       </c>
@@ -797,11 +1898,11 @@
       <c r="K11" s="8">
         <v>0</v>
       </c>
-      <c r="L11" s="12">
+      <c r="L11" s="10">
         <v>0.60037673493920196</v>
       </c>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B12" s="6">
         <v>2000</v>
       </c>
@@ -832,11 +1933,11 @@
       <c r="K12" s="8">
         <v>0</v>
       </c>
-      <c r="L12" s="12">
+      <c r="L12" s="10">
         <v>0.85657363262286745</v>
       </c>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
       <c r="E13" s="8"/>
       <c r="F13" s="8"/>
       <c r="G13" s="8"/>
@@ -844,9 +1945,9 @@
       <c r="I13" s="8"/>
       <c r="J13" s="8"/>
       <c r="K13" s="8"/>
-      <c r="L13" s="12"/>
-    </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="L13" s="10"/>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B14" s="6">
         <v>2500</v>
       </c>
@@ -877,11 +1978,11 @@
       <c r="K14" s="8">
         <v>0</v>
       </c>
-      <c r="L14" s="12">
+      <c r="L14" s="10">
         <v>0.68715767025752461</v>
       </c>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B15" s="6">
         <v>2500</v>
       </c>
@@ -912,11 +2013,11 @@
       <c r="K15" s="8">
         <v>0</v>
       </c>
-      <c r="L15" s="12">
+      <c r="L15" s="10">
         <v>0.90944657866752976</v>
       </c>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
       <c r="E16" s="8"/>
       <c r="F16" s="8"/>
       <c r="G16" s="8"/>
@@ -924,9 +2025,9 @@
       <c r="I16" s="8"/>
       <c r="J16" s="8"/>
       <c r="K16" s="8"/>
-      <c r="L16" s="12"/>
-    </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="L16" s="10"/>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B17" s="6">
         <v>3000</v>
       </c>
@@ -957,11 +2058,11 @@
       <c r="K17" s="8">
         <v>0</v>
       </c>
-      <c r="L17" s="12">
+      <c r="L17" s="10">
         <v>0.74973443524897121</v>
       </c>
     </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B18" s="6">
         <v>3000</v>
       </c>
@@ -992,11 +2093,11 @@
       <c r="K18" s="8">
         <v>0</v>
       </c>
-      <c r="L18" s="12">
+      <c r="L18" s="10">
         <v>0.93713888760460495</v>
       </c>
     </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A19" s="5" t="s">
         <v>13</v>
       </c>
@@ -1007,9 +2108,9 @@
       <c r="I19" s="8"/>
       <c r="J19" s="8"/>
       <c r="K19" s="8"/>
-      <c r="L19" s="12"/>
-    </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="L19" s="10"/>
+    </row>
+    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B20" s="6">
         <v>2500</v>
       </c>
@@ -1040,11 +2141,11 @@
       <c r="K20" s="8">
         <v>2.3400000000000001E-2</v>
       </c>
-      <c r="L20" s="12">
+      <c r="L20" s="10">
         <v>0.70972303480831711</v>
       </c>
     </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B21" s="6">
         <v>2500</v>
       </c>
@@ -1075,11 +2176,11 @@
       <c r="K21" s="8">
         <v>0.25580000000000003</v>
       </c>
-      <c r="L21" s="12">
+      <c r="L21" s="10">
         <v>0.88391302665677118</v>
       </c>
     </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A22" s="5" t="s">
         <v>14</v>
       </c>
@@ -1090,9 +2191,9 @@
       <c r="I22" s="8"/>
       <c r="J22" s="8"/>
       <c r="K22" s="8"/>
-      <c r="L22" s="12"/>
-    </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="L22" s="10"/>
+    </row>
+    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B23" s="6">
         <v>2500</v>
       </c>
@@ -1123,11 +2224,11 @@
       <c r="K23" s="8">
         <v>2.7400000000000001E-2</v>
       </c>
-      <c r="L23" s="12">
+      <c r="L23" s="10">
         <v>0.61690965973230127</v>
       </c>
     </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B24" s="6">
         <v>2500</v>
       </c>
@@ -1158,11 +2259,11 @@
       <c r="K24" s="8">
         <v>0.1178</v>
       </c>
-      <c r="L24" s="12">
+      <c r="L24" s="10">
         <v>0.74325424608934043</v>
       </c>
     </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A25" s="5" t="s">
         <v>15</v>
       </c>
@@ -1173,9 +2274,9 @@
       <c r="I25" s="8"/>
       <c r="J25" s="8"/>
       <c r="K25" s="8"/>
-      <c r="L25" s="12"/>
-    </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="L25" s="10"/>
+    </row>
+    <row r="26" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B26" s="6">
         <v>2500</v>
       </c>
@@ -1206,11 +2307,11 @@
       <c r="K26" s="8">
         <v>0.1244</v>
       </c>
-      <c r="L26" s="12">
+      <c r="L26" s="10">
         <v>0.25319999999999998</v>
       </c>
     </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B27" s="6">
         <v>2500</v>
       </c>
@@ -1241,11 +2342,11 @@
       <c r="K27" s="8">
         <v>4.9000000000000002E-2</v>
       </c>
-      <c r="L27" s="12">
+      <c r="L27" s="10">
         <v>3.1800000000000002E-2</v>
       </c>
     </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A28" s="5" t="s">
         <v>16</v>
       </c>
@@ -1256,9 +2357,9 @@
       <c r="I28" s="8"/>
       <c r="J28" s="8"/>
       <c r="K28" s="8"/>
-      <c r="L28" s="12"/>
-    </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="L28" s="10"/>
+    </row>
+    <row r="29" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B29" s="6">
         <v>2500</v>
       </c>
@@ -1289,11 +2390,11 @@
       <c r="K29" s="8">
         <v>0.12820000000000001</v>
       </c>
-      <c r="L29" s="12">
+      <c r="L29" s="10">
         <v>0.87160000000000004</v>
       </c>
     </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B30" s="6">
         <v>2500</v>
       </c>
@@ -1324,11 +2425,11 @@
       <c r="K30" s="8">
         <v>9.8000000000000004E-2</v>
       </c>
-      <c r="L30" s="12">
+      <c r="L30" s="10">
         <v>0.73140000000000005</v>
       </c>
     </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A31" s="5" t="s">
         <v>17</v>
       </c>
@@ -1339,9 +2440,9 @@
       <c r="I31" s="8"/>
       <c r="J31" s="8"/>
       <c r="K31" s="8"/>
-      <c r="L31" s="12"/>
-    </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="L31" s="10"/>
+    </row>
+    <row r="32" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B32" s="6">
         <v>2500</v>
       </c>
@@ -1372,11 +2473,11 @@
       <c r="K32" s="8">
         <v>7.5399999999999995E-2</v>
       </c>
-      <c r="L32" s="12">
+      <c r="L32" s="10">
         <v>0.29478187931339578</v>
       </c>
     </row>
-    <row r="33" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B33" s="6">
         <v>2500</v>
       </c>
@@ -1407,11 +2508,11 @@
       <c r="K33" s="8">
         <v>9.6799999999999997E-2</v>
       </c>
-      <c r="L33" s="12">
+      <c r="L33" s="10">
         <v>0.13620488409131129</v>
       </c>
     </row>
-    <row r="34" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A34" s="5" t="s">
         <v>18</v>
       </c>
@@ -1422,9 +2523,9 @@
       <c r="I34" s="8"/>
       <c r="J34" s="8"/>
       <c r="K34" s="8"/>
-      <c r="L34" s="12"/>
-    </row>
-    <row r="35" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="L34" s="10"/>
+    </row>
+    <row r="35" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B35" s="6">
         <v>2500</v>
       </c>
@@ -1455,11 +2556,11 @@
       <c r="K35" s="8">
         <v>6.7799999999999999E-2</v>
       </c>
-      <c r="L35" s="12">
+      <c r="L35" s="10">
         <v>0.78614059485646104</v>
       </c>
     </row>
-    <row r="36" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B36" s="6">
         <v>2500</v>
       </c>
@@ -1490,7 +2591,7 @@
       <c r="K36" s="8">
         <v>0.23680000000000001</v>
       </c>
-      <c r="L36" s="12">
+      <c r="L36" s="10">
         <v>0.86776893463479166</v>
       </c>
     </row>

</xml_diff>